<commit_message>
tests: add non-local data for new imports
Adding PbtO2 data, Marshall and IMPACT scores to test data, in order to make the non-local tests running.
</commit_message>
<xml_diff>
--- a/oxytcmri/test-data/outcomes.xlsx
+++ b/oxytcmri/test-data/outcomes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/PSL/NextCloud Leviia/01 - Projets/IRM Oxy-TC/oxytcmri/oxytcmri/test-data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2EFF71B-1FC5-814E-B44F-A74A03CB9017}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE88AF47-0232-8549-8B1B-C2F0BD62E374}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4940" yWindow="1360" windowWidth="22160" windowHeight="14540" xr2:uid="{0AA185AD-772B-674F-9DF0-22933BBDD6EF}"/>
+    <workbookView xWindow="3440" yWindow="1360" windowWidth="22160" windowHeight="14540" xr2:uid="{0AA185AD-772B-674F-9DF0-22933BBDD6EF}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="22">
   <si>
     <t>id_secondaire</t>
   </si>
@@ -78,25 +78,43 @@
   </si>
   <si>
     <t>GOSE_12M</t>
+  </si>
+  <si>
+    <t>impact_mort_ext_pred</t>
+  </si>
+  <si>
+    <t>impact_cfuo_ext_pred</t>
+  </si>
+  <si>
+    <t>tdmadm_marshall_score</t>
+  </si>
+  <si>
+    <t>Hématome massif non évacué</t>
+  </si>
+  <si>
+    <t>II</t>
+  </si>
+  <si>
+    <t>Chirurgie d'évacuation d'hématome</t>
+  </si>
+  <si>
+    <t>I</t>
+  </si>
+  <si>
+    <t/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF6AAB73"/>
-      <name val="JetBrains Mono"/>
-      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -119,10 +137,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -437,249 +456,463 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AEB42E3B-23FA-DC43-BC85-14EF9C0827B1}">
-  <dimension ref="A1:C23"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <dimension ref="A1:F26"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="4" max="4" width="20.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
+      <c r="D1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="3">
         <v>4</v>
       </c>
-      <c r="C2" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="s">
+      <c r="C2" s="3">
+        <v>3</v>
+      </c>
+      <c r="D2" s="1">
+        <v>0.23272281757379898</v>
+      </c>
+      <c r="E2" s="1">
+        <v>0.43118941896080382</v>
+      </c>
+      <c r="F2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="3">
         <v>6</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="3">
         <v>6</v>
       </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" t="s">
+      <c r="D3" s="1">
+        <v>0.30725158258616958</v>
+      </c>
+      <c r="E3" s="1">
+        <v>0.7444066969676133</v>
+      </c>
+      <c r="F3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" s="3">
         <v>5</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="3">
         <v>6</v>
       </c>
-    </row>
-    <row r="5" spans="1:3">
-      <c r="A5" t="s">
+      <c r="D4" s="1">
+        <v>0.21959981133472342</v>
+      </c>
+      <c r="E4" s="1">
+        <v>0.52921667867531819</v>
+      </c>
+      <c r="F4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5" s="3">
         <v>5</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C5" s="3">
         <v>5</v>
       </c>
-    </row>
-    <row r="6" spans="1:3">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="2">
-        <v>3</v>
-      </c>
-      <c r="C6" s="2">
+      <c r="D5" s="1">
+        <v>0.52971494216539605</v>
+      </c>
+      <c r="E5" s="1">
+        <v>0.59676406572544638</v>
+      </c>
+      <c r="F5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="3">
+        <v>3</v>
+      </c>
+      <c r="C6" s="3">
         <v>4</v>
       </c>
-    </row>
-    <row r="7" spans="1:3">
-      <c r="A7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" s="2">
+      <c r="D6" s="1">
+        <v>0.27012272713050861</v>
+      </c>
+      <c r="E6" s="1"/>
+      <c r="F6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="3">
         <v>4</v>
       </c>
-      <c r="C7" s="2">
+      <c r="C7" s="3">
         <v>6</v>
       </c>
-    </row>
-    <row r="8" spans="1:3">
-      <c r="A8" t="s">
+      <c r="D7" s="1">
+        <v>0.20294316871114162</v>
+      </c>
+      <c r="E7" s="1"/>
+      <c r="F7" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A8" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="2">
+      <c r="B8" s="3">
         <v>8</v>
       </c>
-      <c r="C8" s="2">
+      <c r="C8" s="3">
         <v>7</v>
       </c>
-    </row>
-    <row r="9" spans="1:3">
-      <c r="A9" t="s">
+      <c r="D8" s="1">
+        <v>9.1787688339495313E-2</v>
+      </c>
+      <c r="E8" s="1">
+        <v>0.52098766070653224</v>
+      </c>
+      <c r="F8" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="2">
-        <v>3</v>
-      </c>
-      <c r="C9" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3">
-      <c r="A10" t="s">
+      <c r="B9" s="3">
+        <v>3</v>
+      </c>
+      <c r="C9" s="3">
+        <v>3</v>
+      </c>
+      <c r="D9" s="1">
+        <v>0.50824925139402322</v>
+      </c>
+      <c r="E9" s="1">
+        <v>0.86506366140844571</v>
+      </c>
+      <c r="F9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B10" s="2">
+      <c r="B10" s="3">
         <v>4</v>
       </c>
-      <c r="C10" s="2">
+      <c r="C10" s="3">
         <v>7</v>
       </c>
-    </row>
-    <row r="11" spans="1:3">
-      <c r="A11" t="s">
+      <c r="D10" s="1">
+        <v>0.17122077488442922</v>
+      </c>
+      <c r="E10" s="1">
+        <v>0.57615282677128876</v>
+      </c>
+      <c r="F10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A11" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-    </row>
-    <row r="12" spans="1:3">
-      <c r="A12" t="s">
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="1">
+        <v>0.18542741929298232</v>
+      </c>
+      <c r="E11" s="1">
+        <v>0.78414718917748527</v>
+      </c>
+      <c r="F11" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A12" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B12" s="2">
+      <c r="B12" s="3">
         <v>6</v>
       </c>
-      <c r="C12" s="2">
+      <c r="C12" s="3">
         <v>7</v>
       </c>
-    </row>
-    <row r="13" spans="1:3">
-      <c r="A13" t="s">
+      <c r="D12" s="1">
+        <v>0.37754066879814541</v>
+      </c>
+      <c r="E12" s="1">
+        <v>0.63320706348158473</v>
+      </c>
+      <c r="F12" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A13" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B13" s="2">
+      <c r="B13" s="3">
         <v>6</v>
       </c>
-      <c r="C13" s="2">
+      <c r="C13" s="3">
         <v>6</v>
       </c>
-    </row>
-    <row r="14" spans="1:3">
-      <c r="A14" t="s">
+      <c r="D13" s="1">
+        <v>0.26269654621644078</v>
+      </c>
+      <c r="E13" s="1">
+        <v>0.82678341207176609</v>
+      </c>
+      <c r="F13" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A14" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B14" s="2">
-        <v>3</v>
-      </c>
-      <c r="C14" s="2"/>
-    </row>
-    <row r="15" spans="1:3">
-      <c r="A15" t="s">
+      <c r="B14" s="3">
+        <v>3</v>
+      </c>
+      <c r="C14" s="3"/>
+      <c r="D14" s="1">
+        <v>0.36865295576584789</v>
+      </c>
+      <c r="E14" s="1">
+        <v>0.71748086591566318</v>
+      </c>
+      <c r="F14" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A15" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B15" s="2">
+      <c r="B15" s="3">
         <v>5</v>
       </c>
-      <c r="C15" s="2">
+      <c r="C15" s="3">
         <v>5</v>
       </c>
-    </row>
-    <row r="16" spans="1:3">
-      <c r="A16" t="s">
+      <c r="D15" s="1">
+        <v>0.27607804342710862</v>
+      </c>
+      <c r="E15" s="1"/>
+      <c r="F15" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A16" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B16" s="2">
+      <c r="B16" s="3">
         <v>5</v>
       </c>
-      <c r="C16" s="2">
+      <c r="C16" s="3">
         <v>5</v>
       </c>
-    </row>
-    <row r="17" spans="1:3">
-      <c r="A17" t="s">
+      <c r="D16" s="1"/>
+      <c r="E16" s="1">
+        <v>0.33026206907282918</v>
+      </c>
+      <c r="F16" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A17" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-    </row>
-    <row r="18" spans="1:3">
-      <c r="A18" t="s">
+      <c r="B17" s="3"/>
+      <c r="C17" s="3"/>
+      <c r="D17" s="1">
+        <v>0.30959786210964241</v>
+      </c>
+      <c r="E17" s="1">
+        <v>0.83019360535203102</v>
+      </c>
+      <c r="F17" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A18" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B18" s="2">
+      <c r="B18" s="3">
         <v>5</v>
       </c>
-      <c r="C18" s="2">
+      <c r="C18" s="3">
         <v>7</v>
       </c>
-    </row>
-    <row r="19" spans="1:3">
-      <c r="A19" t="s">
+      <c r="D18" s="1">
+        <v>0.35183111816157903</v>
+      </c>
+      <c r="E18" s="1">
+        <v>0.364705150677193</v>
+      </c>
+      <c r="F18" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A19" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B19" s="2">
+      <c r="B19" s="3">
         <v>1</v>
       </c>
-      <c r="C19" s="2">
+      <c r="C19" s="3">
         <v>1</v>
       </c>
-    </row>
-    <row r="20" spans="1:3">
-      <c r="A20" t="s">
+      <c r="D19" s="1">
+        <v>0.93388761453661562</v>
+      </c>
+      <c r="E19" s="1">
+        <v>0.62128359519106779</v>
+      </c>
+      <c r="F19" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A20" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B20" s="2">
-        <v>3</v>
-      </c>
-      <c r="C20" s="2">
+      <c r="B20" s="3">
+        <v>3</v>
+      </c>
+      <c r="C20" s="3">
         <v>4</v>
       </c>
-    </row>
-    <row r="21" spans="1:3">
-      <c r="A21" t="s">
+      <c r="D20" s="1">
+        <v>0.49900000133333117</v>
+      </c>
+      <c r="E20" s="1">
+        <v>0.69656633303768789</v>
+      </c>
+      <c r="F20" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A21" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B21" s="2">
+      <c r="B21" s="3">
         <v>4</v>
       </c>
-      <c r="C21" s="2"/>
-    </row>
-    <row r="22" spans="1:3">
-      <c r="A22" t="s">
+      <c r="C21" s="3"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1">
+        <v>0.91364694192489748</v>
+      </c>
+      <c r="F21" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A22" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B22" s="2">
-        <v>3</v>
-      </c>
-      <c r="C22" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3">
-      <c r="A23" t="s">
+      <c r="B22" s="3">
+        <v>3</v>
+      </c>
+      <c r="C22" s="3">
+        <v>3</v>
+      </c>
+      <c r="D22" s="1">
+        <v>0.50599971201658789</v>
+      </c>
+      <c r="E22" s="1">
+        <v>0.73846392043063558</v>
+      </c>
+      <c r="F22" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A23" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B23" s="2">
-        <v>3</v>
-      </c>
-      <c r="C23" s="2">
+      <c r="B23" s="3">
+        <v>3</v>
+      </c>
+      <c r="C23" s="3">
         <v>4</v>
       </c>
+      <c r="D23" s="1">
+        <v>0.30597597335744869</v>
+      </c>
+      <c r="E23" s="1">
+        <v>0.41872733339077445</v>
+      </c>
+      <c r="F23" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="D24" s="1"/>
+      <c r="E24" s="1"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="D25" s="1"/>
+      <c r="E25" s="1"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="D26" s="1"/>
+      <c r="E26" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>